<commit_message>
finished schematic for phase 90 and implemented the correct op-amps for overdrive
</commit_message>
<xml_diff>
--- a/phase90/JFET characterization/jfet characterization.xlsx
+++ b/phase90/JFET characterization/jfet characterization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Desktop\ECE 4014\RGA\RGA_Boards\phase90\JFET characterization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D431713-E92F-417B-8FBC-E1AAAC05BEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B34F56-DA2A-4CE7-9839-97E264AEBFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,13 +59,13 @@
     <t>Vout (mV)</t>
   </si>
   <si>
-    <t>Rdson2</t>
-  </si>
-  <si>
     <t>Idss (mA)</t>
   </si>
   <si>
     <t>Rgs1</t>
+  </si>
+  <si>
+    <t>Rdson</t>
   </si>
 </sst>
 </file>
@@ -81,12 +81,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -101,13 +119,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -139,22 +164,24 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9B547DEC-811B-4E63-A80F-AB8FCAA9868D}" name="JFET number"/>
     <tableColumn id="2" xr3:uid="{0388F1F5-6784-4F51-9BE0-DD0D4B2E34F4}" name="Idss (mA)"/>
-    <tableColumn id="10" xr3:uid="{4F3BEE6B-9395-40E7-8758-EBF4E3CA9B48}" name="Vgs1" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{4F3BEE6B-9395-40E7-8758-EBF4E3CA9B48}" name="Vgs1" dataDxfId="4">
       <calculatedColumnFormula>0-15+G2*D2*0.001</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{EA397B9A-768D-425D-AFB5-214A5302FDA8}" name="Rgs1"/>
     <tableColumn id="4" xr3:uid="{34AB69A6-4FA6-4DE0-B121-6C932A717D84}" name="Beta" dataDxfId="3">
       <calculatedColumnFormula>B2/(4*D2*D2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B3D0C7AD-ECDE-4382-9AEE-EF201B4C1419}" name="Vto" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{B3D0C7AD-ECDE-4382-9AEE-EF201B4C1419}" name="Vto" dataDxfId="2">
       <calculatedColumnFormula>2*D2*0.001</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{90732221-72A7-4750-8472-FD912D897A39}" name="Idss/4 (mA)" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{90732221-72A7-4750-8472-FD912D897A39}" name="Idss/4 (mA)" dataDxfId="1">
       <calculatedColumnFormula>B2/4</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{F74B3BEF-DD30-42A9-B3CA-26DA01E88213}" name="Vin (mV)"/>
     <tableColumn id="8" xr3:uid="{ED07ED67-59A7-4C04-AB09-63E7F88307EE}" name="Vout (mV)"/>
-    <tableColumn id="9" xr3:uid="{724CB172-CA09-4430-8A5A-0D31ACF205E1}" name="Rdson2"/>
+    <tableColumn id="9" xr3:uid="{724CB172-CA09-4430-8A5A-0D31ACF205E1}" name="Rdson" dataDxfId="0">
+      <calculatedColumnFormula>510*I2/(H2-I2)</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -429,7 +456,7 @@
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="3" width="14.6640625" customWidth="1"/>
     <col min="4" max="4" width="11.88671875" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" customWidth="1"/>
     <col min="8" max="8" width="14.109375" customWidth="1"/>
@@ -442,13 +469,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -466,34 +493,38 @@
         <v>6</v>
       </c>
       <c r="J1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>7.92</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="2">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="C2" s="2">
         <f t="shared" ref="C2:C21" si="0">0-15+G2*D2*0.001</f>
-        <v>-13.98624</v>
-      </c>
-      <c r="D2">
-        <v>512</v>
-      </c>
-      <c r="E2">
+        <v>-13.516375</v>
+      </c>
+      <c r="D2" s="2">
+        <v>715</v>
+      </c>
+      <c r="E2" s="2">
         <f t="shared" ref="E2:E21" si="1">B2/(4*D2*D2)</f>
-        <v>7.5531005859374999E-6</v>
-      </c>
-      <c r="F2">
+        <v>4.0588781847523108E-6</v>
+      </c>
+      <c r="F2" s="2">
         <f t="shared" ref="F2:F21" si="2">2*D2*0.001</f>
-        <v>1.024</v>
-      </c>
-      <c r="G2">
+        <v>1.43</v>
+      </c>
+      <c r="G2" s="2">
         <f t="shared" ref="G2:G21" si="3">B2/4</f>
-        <v>1.98</v>
+        <v>2.0750000000000002</v>
+      </c>
+      <c r="J2" s="2" t="e">
+        <f t="shared" ref="J2:J21" si="4">510*I2/(H2-I2)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -501,161 +532,197 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>9.41</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <f t="shared" si="0"/>
-        <v>-13.807282499999999</v>
+        <v>-13.29</v>
       </c>
       <c r="D3">
-        <v>507</v>
+        <v>684</v>
       </c>
       <c r="E3">
         <f t="shared" si="1"/>
-        <v>9.1519515734354158E-6</v>
+        <v>5.3435245032659618E-6</v>
       </c>
       <c r="F3">
         <f t="shared" si="2"/>
-        <v>1.014</v>
+        <v>1.3680000000000001</v>
       </c>
       <c r="G3">
         <f t="shared" si="3"/>
-        <v>2.3525</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4">
+        <v>2.5</v>
+      </c>
+      <c r="J3" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>8.7309999999999999</v>
-      </c>
-      <c r="C4">
-        <f t="shared" si="0"/>
-        <v>-13.873701000000001</v>
-      </c>
-      <c r="D4">
-        <v>516</v>
-      </c>
-      <c r="E4">
-        <f t="shared" si="1"/>
-        <v>8.1979373234781567E-6</v>
-      </c>
-      <c r="F4">
-        <f t="shared" si="2"/>
-        <v>1.032</v>
-      </c>
-      <c r="G4">
-        <f t="shared" si="3"/>
-        <v>2.18275</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
+      <c r="B4" s="1">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="shared" si="0"/>
+        <v>-13.378500000000001</v>
+      </c>
+      <c r="D4" s="1">
+        <v>705</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="1"/>
+        <v>4.6275338262662841E-6</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="2"/>
+        <v>1.41</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="3"/>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="J4" s="1" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>8.68</v>
-      </c>
-      <c r="C5">
-        <f t="shared" si="0"/>
-        <v>-13.880279999999999</v>
-      </c>
-      <c r="D5">
-        <v>516</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
-        <v>8.1500510786611371E-6</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="2"/>
-        <v>1.032</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="3"/>
-        <v>2.17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6">
+      <c r="B5" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="shared" si="0"/>
+        <v>-13.396125</v>
+      </c>
+      <c r="D5" s="1">
+        <v>705</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="1"/>
+        <v>4.5772345455459985E-6</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="2"/>
+        <v>1.41</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="3"/>
+        <v>2.2749999999999999</v>
+      </c>
+      <c r="J5" s="1" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>8.173</v>
-      </c>
-      <c r="C6">
-        <f t="shared" si="0"/>
-        <v>-13.947726250000001</v>
-      </c>
-      <c r="D6">
-        <v>515</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
-        <v>7.7038363653501748E-6</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="2"/>
-        <v>1.03</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="3"/>
-        <v>2.04325</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7">
+      <c r="B6" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="C6" s="2">
+        <f t="shared" si="0"/>
+        <v>-13.480625</v>
+      </c>
+      <c r="D6" s="2">
+        <v>715</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" si="1"/>
+        <v>4.1566824783608002E-6</v>
+      </c>
+      <c r="F6" s="2">
+        <f t="shared" si="2"/>
+        <v>1.43</v>
+      </c>
+      <c r="G6" s="2">
+        <f t="shared" si="3"/>
+        <v>2.125</v>
+      </c>
+      <c r="H6" s="2">
+        <v>188</v>
+      </c>
+      <c r="I6" s="2">
+        <v>46</v>
+      </c>
+      <c r="J6" s="2">
+        <f t="shared" si="4"/>
+        <v>165.21126760563379</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>7.9749999999999996</v>
-      </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
-        <v>-13.971225</v>
-      </c>
-      <c r="D7">
-        <v>516</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
-        <v>7.4880941650141211E-6</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="2"/>
-        <v>1.032</v>
-      </c>
-      <c r="G7">
-        <f t="shared" si="3"/>
-        <v>1.9937499999999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8">
+      <c r="B7" s="3">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="C7" s="3">
+        <f t="shared" si="0"/>
+        <v>-13.499775</v>
+      </c>
+      <c r="D7" s="3">
+        <v>723</v>
+      </c>
+      <c r="E7" s="3">
+        <f t="shared" si="1"/>
+        <v>3.9695521006104503E-6</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="2"/>
+        <v>1.446</v>
+      </c>
+      <c r="G7" s="3">
+        <f t="shared" si="3"/>
+        <v>2.0750000000000002</v>
+      </c>
+      <c r="H7" s="3">
+        <v>188</v>
+      </c>
+      <c r="I7" s="3">
+        <v>47</v>
+      </c>
+      <c r="J7" s="3">
+        <f t="shared" si="4"/>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>8.1150000000000002</v>
-      </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
-        <v>-13.953165</v>
-      </c>
-      <c r="D8">
-        <v>516</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
-        <v>7.6195466017667211E-6</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="2"/>
-        <v>1.032</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="3"/>
-        <v>2.0287500000000001</v>
+      <c r="B8" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="C8" s="3">
+        <f t="shared" si="0"/>
+        <v>-13.463625</v>
+      </c>
+      <c r="D8" s="3">
+        <v>723</v>
+      </c>
+      <c r="E8" s="3">
+        <f t="shared" si="1"/>
+        <v>4.0652039584564853E-6</v>
+      </c>
+      <c r="F8" s="3">
+        <f t="shared" si="2"/>
+        <v>1.446</v>
+      </c>
+      <c r="G8" s="3">
+        <f t="shared" si="3"/>
+        <v>2.125</v>
+      </c>
+      <c r="J8" s="3" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -663,26 +730,30 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>7.0049999999999999</v>
+        <v>7.25</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>-14.094603749999999</v>
+        <v>-13.666</v>
       </c>
       <c r="D9">
-        <v>517</v>
+        <v>736</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
-        <v>6.5518970103520911E-6</v>
+        <v>3.3459726488657847E-6</v>
       </c>
       <c r="F9">
         <f t="shared" si="2"/>
-        <v>1.034</v>
+        <v>1.472</v>
       </c>
       <c r="G9">
         <f t="shared" si="3"/>
-        <v>1.75125</v>
+        <v>1.8125</v>
+      </c>
+      <c r="J9" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -690,275 +761,377 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>7.2889999999999997</v>
+        <v>7.6</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>-14.061541249999999</v>
+        <v>-13.6282</v>
       </c>
       <c r="D10">
-        <v>515</v>
+        <v>722</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
-        <v>6.8705815816759356E-6</v>
+        <v>3.6448461874908875E-6</v>
       </c>
       <c r="F10">
         <f t="shared" si="2"/>
-        <v>1.03</v>
+        <v>1.444</v>
       </c>
       <c r="G10">
         <f t="shared" si="3"/>
-        <v>1.8222499999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11">
+        <v>1.9</v>
+      </c>
+      <c r="J10" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11">
-        <v>8.33</v>
-      </c>
-      <c r="C11">
-        <f t="shared" si="0"/>
-        <v>-13.931677499999999</v>
-      </c>
-      <c r="D11">
-        <v>513</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="1"/>
-        <v>7.9131660643920827E-6</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="2"/>
-        <v>1.026</v>
-      </c>
-      <c r="G11">
-        <f t="shared" si="3"/>
-        <v>2.0825</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12">
+      <c r="B11" s="1">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="C11" s="1">
+        <f t="shared" si="0"/>
+        <v>-13.4688</v>
+      </c>
+      <c r="D11" s="1">
+        <v>696</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="1"/>
+        <v>4.5415510635486858E-6</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="2"/>
+        <v>1.3920000000000001</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="3"/>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="J11" s="1" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>8.0559999999999992</v>
-      </c>
-      <c r="C12">
-        <f t="shared" si="0"/>
-        <v>-13.966818</v>
-      </c>
-      <c r="D12">
-        <v>513</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="1"/>
-        <v>7.6528770485885488E-6</v>
-      </c>
-      <c r="F12">
-        <f t="shared" si="2"/>
-        <v>1.026</v>
-      </c>
-      <c r="G12">
-        <f t="shared" si="3"/>
-        <v>2.0139999999999998</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13">
+      <c r="B12" s="2">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="C12" s="2">
+        <f t="shared" si="0"/>
+        <v>-13.4980125</v>
+      </c>
+      <c r="D12" s="2">
+        <v>711</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="1"/>
+        <v>4.1788570603397284E-6</v>
+      </c>
+      <c r="F12" s="2">
+        <f t="shared" si="2"/>
+        <v>1.4219999999999999</v>
+      </c>
+      <c r="G12" s="2">
+        <f t="shared" si="3"/>
+        <v>2.1124999999999998</v>
+      </c>
+      <c r="J12" s="2" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>8.2170000000000005</v>
-      </c>
-      <c r="C13">
-        <f t="shared" si="0"/>
-        <v>-13.944115500000001</v>
-      </c>
-      <c r="D13">
-        <v>514</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="1"/>
-        <v>7.7754772971581712E-6</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="2"/>
-        <v>1.028</v>
-      </c>
-      <c r="G13">
-        <f t="shared" si="3"/>
-        <v>2.0542500000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14">
+      <c r="B13" s="2">
+        <v>8.6</v>
+      </c>
+      <c r="C13" s="2">
+        <f t="shared" si="0"/>
+        <v>-13.456300000000001</v>
+      </c>
+      <c r="D13" s="2">
+        <v>718</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="1"/>
+        <v>4.170513884901576E-6</v>
+      </c>
+      <c r="F13" s="2">
+        <f t="shared" si="2"/>
+        <v>1.4359999999999999</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" si="3"/>
+        <v>2.15</v>
+      </c>
+      <c r="J13" s="2" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="C14">
-        <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E14" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F14">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <f t="shared" si="3"/>
-        <v>0</v>
+      <c r="B14" s="1">
+        <v>8.9</v>
+      </c>
+      <c r="C14" s="1">
+        <f t="shared" si="0"/>
+        <v>-13.4336</v>
+      </c>
+      <c r="D14" s="1">
+        <v>704</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="1"/>
+        <v>4.4893627324380165E-6</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="2"/>
+        <v>1.4079999999999999</v>
+      </c>
+      <c r="G14" s="1">
+        <f t="shared" si="3"/>
+        <v>2.2250000000000001</v>
+      </c>
+      <c r="H14" s="1">
+        <v>188</v>
+      </c>
+      <c r="I14" s="1">
+        <v>46</v>
+      </c>
+      <c r="J14" s="1">
+        <f t="shared" si="4"/>
+        <v>165.21126760563379</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
+      <c r="B15">
+        <v>9.9</v>
+      </c>
       <c r="C15">
         <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E15" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-13.299675000000001</v>
+      </c>
+      <c r="D15">
+        <v>687</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="1"/>
+        <v>5.2439884822943885E-6</v>
       </c>
       <c r="F15">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.3740000000000001</v>
       </c>
       <c r="G15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.4750000000000001</v>
+      </c>
+      <c r="J15" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
+      <c r="B16">
+        <v>10</v>
+      </c>
       <c r="C16">
         <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E16" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-13.29</v>
+      </c>
+      <c r="D16">
+        <v>684</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="1"/>
+        <v>5.3435245032659618E-6</v>
       </c>
       <c r="F16">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.3680000000000001</v>
       </c>
       <c r="G16">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17">
+        <v>2.5</v>
+      </c>
+      <c r="J16" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="C17">
-        <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E17" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F17">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B17" s="3">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C17" s="3">
+        <f t="shared" si="0"/>
+        <v>-13.524000000000001</v>
+      </c>
+      <c r="D17" s="3">
+        <v>720</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" si="1"/>
+        <v>3.9544753086419754E-6</v>
+      </c>
+      <c r="F17" s="3">
+        <f t="shared" si="2"/>
+        <v>1.44</v>
+      </c>
+      <c r="G17" s="3">
+        <f t="shared" si="3"/>
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="J17" s="3" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
+      <c r="B18">
+        <v>9.5</v>
+      </c>
       <c r="C18">
         <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E18" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-13.327999999999999</v>
+      </c>
+      <c r="D18">
+        <v>704</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>4.7920163997933886E-6</v>
       </c>
       <c r="F18">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.4079999999999999</v>
       </c>
       <c r="G18">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19">
+        <v>2.375</v>
+      </c>
+      <c r="J18" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="C19">
-        <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E19" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F19">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G19">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="4">
+        <v>8.1</v>
+      </c>
+      <c r="C19" s="4">
+        <f t="shared" si="0"/>
+        <v>-13.527825</v>
+      </c>
+      <c r="D19" s="4">
+        <v>727</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" si="1"/>
+        <v>3.8313886276817351E-6</v>
+      </c>
+      <c r="F19" s="4">
+        <f t="shared" si="2"/>
+        <v>1.454</v>
+      </c>
+      <c r="G19" s="4">
+        <f t="shared" si="3"/>
+        <v>2.0249999999999999</v>
+      </c>
+      <c r="J19" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
+      <c r="B20">
+        <v>7.3</v>
+      </c>
       <c r="C20">
         <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E20" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-13.627600000000001</v>
+      </c>
+      <c r="D20">
+        <v>752</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>3.227209710276143E-6</v>
       </c>
       <c r="F20">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.504</v>
       </c>
       <c r="G20">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21">
+        <v>1.825</v>
+      </c>
+      <c r="J20" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="C21">
-        <f t="shared" si="0"/>
-        <v>-15</v>
-      </c>
-      <c r="E21" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F21">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G21">
-        <f t="shared" si="3"/>
-        <v>0</v>
+      <c r="B21" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="C21" s="3">
+        <f t="shared" si="0"/>
+        <v>-13.45725</v>
+      </c>
+      <c r="D21" s="3">
+        <v>726</v>
+      </c>
+      <c r="E21" s="3">
+        <f t="shared" si="1"/>
+        <v>4.0316766462521533E-6</v>
+      </c>
+      <c r="F21" s="3">
+        <f t="shared" si="2"/>
+        <v>1.452</v>
+      </c>
+      <c r="G21" s="3">
+        <f t="shared" si="3"/>
+        <v>2.125</v>
+      </c>
+      <c r="J21" s="3" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>